<commit_message>
unit of measure neverland sets
</commit_message>
<xml_diff>
--- a/hypatia/examples/Neverland/sets/global.xlsx
+++ b/hypatia/examples/Neverland/sets/global.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{3E916677-621C-4DDE-8C11-D68D08E445AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C17CA945-860D-4DC0-BAE2-B46221448E74}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="13_ncr:1_{3E916677-621C-4DDE-8C11-D68D08E445AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F786453E-26F8-48A3-97E6-EA32139852BA}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -197,12 +197,6 @@
     <t>Electricity_demand</t>
   </si>
   <si>
-    <t>kW</t>
-  </si>
-  <si>
-    <t>kWh</t>
-  </si>
-  <si>
     <t>Unit</t>
   </si>
   <si>
@@ -279,6 +273,12 @@
   </si>
   <si>
     <t>Gas</t>
+  </si>
+  <si>
+    <t>GW</t>
+  </si>
+  <si>
+    <t>GWh</t>
   </si>
 </sst>
 </file>
@@ -434,6 +434,208 @@
   </cellStyles>
   <dxfs count="30">
     <dxf>
+      <numFmt numFmtId="164" formatCode="0.0000000000"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -463,208 +665,6 @@
           <color indexed="64"/>
         </vertical>
         <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0000000000"/>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -903,34 +903,34 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Regions" displayName="Regions" ref="A1:B3" totalsRowShown="0">
   <autoFilter ref="A1:B3" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Region" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Region_name" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Region" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Region_name" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Technologies_glob" displayName="Technologies_glob" ref="A13:E21" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Technologies_glob" displayName="Technologies_glob" ref="A13:E21" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11" totalsRowBorderDxfId="10">
   <autoFilter ref="A13:E21" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="5">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Technology" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Tech_name" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Tech_category" dataDxfId="9"/>
-    <tableColumn id="1" xr3:uid="{F7E6113B-7421-48DB-83C7-8FFAA984C463}" name="Tech_cap_unit" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{3B7F032B-74C4-4B96-86A6-79EEAB4503A1}" name="Tech_act_unit" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Technology" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Tech_name" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Tech_category" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{F7E6113B-7421-48DB-83C7-8FFAA984C463}" name="Tech_cap_unit" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{3B7F032B-74C4-4B96-86A6-79EEAB4503A1}" name="Tech_act_unit" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Timesteps" displayName="Timesteps" ref="A31:C55" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Timesteps" displayName="Timesteps" ref="A31:C55" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="A31:C55" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Timeslice" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Timeslice_name" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Timeslice_fraction" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Timeslice" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Timeslice_name" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Timeslice_fraction" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1253,7 +1253,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>2</v>
@@ -1273,13 +1273,13 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>73</v>
-      </c>
       <c r="D3" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E3" s="6">
         <v>2026</v>
@@ -1287,7 +1287,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D4" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E4" s="6">
         <v>2027</v>
@@ -1295,7 +1295,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D5" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E5" s="6">
         <v>2028</v>
@@ -1303,7 +1303,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D6" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E6" s="6">
         <v>2029</v>
@@ -1311,7 +1311,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D7" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E7" s="6">
         <v>2030</v>
@@ -1319,7 +1319,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D8" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E8" s="6">
         <v>2031</v>
@@ -1327,7 +1327,7 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D9" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E9" s="6">
         <v>2032</v>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D10" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E10" s="6">
         <v>2033</v>
@@ -1343,7 +1343,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="D11" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E11" s="6">
         <v>2034</v>
@@ -1372,121 +1372,121 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>16</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
@@ -1500,10 +1500,10 @@
         <v>8</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
@@ -1527,44 +1527,44 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
@@ -1578,7 +1578,7 @@
         <v>8</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
@@ -1880,15 +1880,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100241E96938535DD4B921FCDFB54345D30" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a684a74f1c6746079667ad43256762fb">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e" xmlns:ns3="e67e9a88-35e1-4b39-8da9-a609eb308282" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb365b527691b54101d88dcd129f0f60" ns2:_="" ns3:_="">
     <xsd:import namespace="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
@@ -2143,6 +2134,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2163,14 +2163,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{400CE890-4FAA-43FF-AB05-78D100D91AC8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F571C89-B126-4182-8FAD-79E7F0190403}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2189,6 +2181,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{400CE890-4FAA-43FF-AB05-78D100D91AC8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82347752-6D50-4565-8A47-C3BD006EDCEE}">
   <ds:schemaRefs>

</xml_diff>